<commit_message>
Add DOM.RF IDs to group workbooks
</commit_message>
<xml_diff>
--- a/_to_delete/приложение по застройщику/Приложение 1  - СЗ ЮНИКС.xlsx
+++ b/_to_delete/приложение по застройщику/Приложение 1  - СЗ ЮНИКС.xlsx
@@ -48,7 +48,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -174,11 +174,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -213,6 +233,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -556,14 +578,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:N6"/>
+  <dimension ref="B2:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.5703125" customWidth="1" min="2" max="2"/>
     <col width="21.140625" customWidth="1" min="3" max="3"/>
     <col width="18.85546875" customWidth="1" min="4" max="4"/>
     <col width="16.7109375" customWidth="1" min="5" max="5"/>
-    <col width="16.5703125" customWidth="1" min="6" max="6"/>
+    <col width="22.85546875" customWidth="1" min="6" max="6"/>
     <col width="22.85546875" customWidth="1" min="7" max="7"/>
     <col width="21.5703125" customWidth="1" min="8" max="8"/>
     <col width="29.42578125" customWidth="1" min="9" max="9"/>
@@ -605,42 +627,43 @@
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
+          <t>id (по данным ЕИСЖС)</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
           <t>№ проектной декларации</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>Количество заключенных ДДУ, ед.</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>Количество исполенных ДДУ, ед.</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="J3" s="11" t="inlineStr">
         <is>
           <t>Первоначальная дата передачи объекта долевого строительства согласно первой проекутной декаларции</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">Текущая дата передачи объекта долевого строительства </t>
         </is>
       </c>
-      <c r="K3" s="11" t="inlineStr">
+      <c r="L3" s="11" t="inlineStr">
         <is>
           <t>Количество ДДУ 
 с переносом срока, ед.</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>из них:</t>
-        </is>
-      </c>
       <c r="M3" s="12" t="n"/>
       <c r="N3" s="13" t="n"/>
+      <c r="O3" s="13" t="n"/>
     </row>
     <row r="4" ht="32.25" customHeight="1">
       <c r="B4" s="14" t="n"/>
@@ -653,13 +676,10 @@
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="n"/>
       <c r="K4" s="14" t="n"/>
-      <c r="L4" s="11" t="inlineStr">
-        <is>
-          <t>Заключено ДС к ДДУ</t>
-        </is>
-      </c>
-      <c r="M4" s="13" t="n"/>
-      <c r="N4" s="11" t="inlineStr">
+      <c r="L4" s="15" t="n"/>
+      <c r="M4" s="17" t="n"/>
+      <c r="N4" s="13" t="n"/>
+      <c r="O4" s="11" t="inlineStr">
         <is>
           <t>не заключено ДС к ДДУ</t>
         </is>
@@ -676,17 +696,14 @@
       <c r="I5" s="15" t="n"/>
       <c r="J5" s="15" t="n"/>
       <c r="K5" s="15" t="n"/>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>количество ДС к ДДУ, ед.</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>дата передачи согласно ДС</t>
-        </is>
-      </c>
-      <c r="N5" s="15" t="n"/>
+      <c r="N5" s="17" t="n"/>
+      <c r="O5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="1" t="inlineStr">
@@ -705,12 +722,16 @@
         </is>
       </c>
       <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>48353</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>77-002758</t>
         </is>
       </c>
-      <c r="G6" s="1" t="n"/>
       <c r="H6" s="1" t="n"/>
       <c r="I6" s="1" t="n"/>
       <c r="J6" s="1" t="n"/>
@@ -718,6 +739,7 @@
       <c r="L6" s="1" t="n"/>
       <c r="M6" s="1" t="n"/>
       <c r="N6" s="1" t="n"/>
+      <c r="O6" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>

<commit_message>
Fix group workbook headers after ID insert
</commit_message>
<xml_diff>
--- a/_to_delete/приложение по застройщику/Приложение 1  - СЗ ЮНИКС.xlsx
+++ b/_to_delete/приложение по застройщику/Приложение 1  - СЗ ЮНИКС.xlsx
@@ -585,22 +585,22 @@
     <col width="21.140625" customWidth="1" min="3" max="3"/>
     <col width="18.85546875" customWidth="1" min="4" max="4"/>
     <col width="16.7109375" customWidth="1" min="5" max="5"/>
-    <col width="22.85546875" customWidth="1" min="6" max="6"/>
-    <col width="22.85546875" customWidth="1" min="7" max="7"/>
-    <col width="21.5703125" customWidth="1" min="8" max="8"/>
-    <col width="29.42578125" customWidth="1" min="9" max="9"/>
-    <col width="31" customWidth="1" min="10" max="10"/>
-    <col width="22.85546875" customWidth="1" min="11" max="11"/>
-    <col width="26.140625" customWidth="1" min="12" max="12"/>
-    <col width="20.85546875" customWidth="1" min="13" max="13"/>
-    <col width="25.42578125" customWidth="1" min="14" max="14"/>
-    <col width="22.85546875" customWidth="1" min="15" max="15"/>
+    <col width="16.5703125" customWidth="1" min="6" max="6"/>
+    <col width="16.5703125" customWidth="1" min="7" max="7"/>
+    <col width="22.85546875" customWidth="1" min="8" max="8"/>
+    <col width="21.5703125" customWidth="1" min="9" max="9"/>
+    <col width="29.42578125" customWidth="1" min="10" max="10"/>
+    <col width="31" customWidth="1" min="11" max="11"/>
+    <col width="22.85546875" customWidth="1" min="12" max="12"/>
+    <col width="26.140625" customWidth="1" min="13" max="13"/>
+    <col width="20.85546875" customWidth="1" min="14" max="14"/>
+    <col width="25.42578125" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Приложение 2 Сроки передачи ключей</t>
+          <t>Приложение 1 Сроки передачи ключей</t>
         </is>
       </c>
     </row>
@@ -661,8 +661,12 @@
 с переносом срока, ед.</t>
         </is>
       </c>
-      <c r="M3" s="12" t="n"/>
-      <c r="N3" s="13" t="n"/>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>из них:</t>
+        </is>
+      </c>
+      <c r="N3" s="12" t="n"/>
       <c r="O3" s="13" t="n"/>
     </row>
     <row r="4" ht="32.25" customHeight="1">
@@ -676,8 +680,12 @@
       <c r="I4" s="14" t="n"/>
       <c r="J4" s="14" t="n"/>
       <c r="K4" s="14" t="n"/>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="17" t="n"/>
+      <c r="L4" s="14" t="n"/>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>Заключено ДС к ДДУ</t>
+        </is>
+      </c>
       <c r="N4" s="13" t="n"/>
       <c r="O4" s="11" t="inlineStr">
         <is>
@@ -702,7 +710,11 @@
           <t>количество ДС к ДДУ, ед.</t>
         </is>
       </c>
-      <c r="N5" s="17" t="n"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>дата передачи согласно ДС</t>
+        </is>
+      </c>
       <c r="O5" s="15" t="n"/>
     </row>
     <row r="6">
@@ -744,18 +756,18 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="H3:H5"/>
-    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L3:L5"/>
+    <mergeCell ref="M3:O3"/>
     <mergeCell ref="C3:C5"/>
-    <mergeCell ref="L3:N3"/>
-    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="D3:D5"/>
     <mergeCell ref="G3:G5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="F3:F5"/>
-    <mergeCell ref="D3:D5"/>
     <mergeCell ref="B3:B5"/>
-    <mergeCell ref="J3:J5"/>
     <mergeCell ref="K3:K5"/>
     <mergeCell ref="I3:I5"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="J3:J5"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="46" fitToHeight="0"/>

</xml_diff>